<commit_message>
Fix Excel template alignment and retain expected sheets
</commit_message>
<xml_diff>
--- a/Safer_City_Test_Cases.xlsx
+++ b/Safer_City_Test_Cases.xlsx
@@ -4,6 +4,7 @@
   <workbookPr/>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crime Reporting Scenarios" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Automation" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -338,7 +339,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="85">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -555,15 +556,12 @@
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -696,7 +694,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table_2" displayName="Table_2" ref="B1:F4" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table_1" displayName="Table_1" ref="B1:F6" headerRowCount="1">
   <tableColumns count="5">
     <tableColumn id="1" name="TEST TITLE"/>
     <tableColumn id="2" name="PRIORITY"/>
@@ -704,7 +702,7 @@
     <tableColumn id="4" name="TEST NUMBER"/>
     <tableColumn id="5" name="TEST DATE"/>
   </tableColumns>
-  <tableStyleInfo name="Registration-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="Partner Uber Login (iOS)-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -906,9 +904,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.75" customWidth="1" style="77" min="2" max="2"/>
@@ -954,355 +952,352 @@
       <c r="I1" s="18" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="18" t="n"/>
-      <c r="B2" s="42" t="inlineStr">
-        <is>
-          <t>EUNIFIN REGISTRATION</t>
-        </is>
-      </c>
-      <c r="C2" s="43" t="inlineStr">
+      <c r="A2" s="78" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="B2" s="79" t="inlineStr">
+        <is>
+          <t>Submit Crime Report with Valid Inputs (End-to-End)</t>
+        </is>
+      </c>
+      <c r="C2" s="78" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D2" s="44" t="inlineStr">
-        <is>
-          <t>#002</t>
-        </is>
-      </c>
-      <c r="E2" s="45" t="n">
-        <v>2</v>
-      </c>
-      <c r="F2" s="46" t="n">
-        <v>46042</v>
-      </c>
-      <c r="G2" s="18" t="n"/>
-      <c r="H2" s="7" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="I2" s="18" t="n"/>
+      <c r="D2" s="79" t="inlineStr">
+        <is>
+          <t>CRF-001</t>
+        </is>
+      </c>
+      <c r="E2" s="78" t="inlineStr">
+        <is>
+          <t>TC-01</t>
+        </is>
+      </c>
+      <c r="F2" s="78" t="inlineStr">
+        <is>
+          <t>26/02/2026</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="n"/>
-      <c r="B3" s="47" t="n"/>
-      <c r="C3" s="47" t="n"/>
-      <c r="D3" s="48" t="inlineStr">
-        <is>
-          <t>TEST DESIGNED BY</t>
-        </is>
-      </c>
-      <c r="E3" s="48" t="inlineStr">
-        <is>
-          <t>TEST EXECUTED BY</t>
-        </is>
-      </c>
-      <c r="F3" s="49" t="inlineStr">
-        <is>
-          <t>EXECUTION DATE</t>
-        </is>
-      </c>
-      <c r="G3" s="18" t="n"/>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="I3" s="18" t="n"/>
+      <c r="A3" s="78" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="B3" s="79" t="inlineStr">
+        <is>
+          <t>Modify Location Details Before Submission</t>
+        </is>
+      </c>
+      <c r="C3" s="78" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D3" s="79" t="inlineStr">
+        <is>
+          <t>CRF-002</t>
+        </is>
+      </c>
+      <c r="E3" s="78" t="inlineStr">
+        <is>
+          <t>TC-02</t>
+        </is>
+      </c>
+      <c r="F3" s="78" t="inlineStr">
+        <is>
+          <t>26/02/2026</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="B4" s="83" t="inlineStr">
-        <is>
-          <t>Submit Crime Report with Valid Inputs (End-to-End)</t>
-        </is>
-      </c>
-      <c r="C4" s="83" t="inlineStr">
+      <c r="A4" s="78" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="B4" s="79" t="inlineStr">
+        <is>
+          <t>Prevent progression with Empty required fields (Step 1)</t>
+        </is>
+      </c>
+      <c r="C4" s="78" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D4" s="84" t="inlineStr">
-        <is>
-          <t>CRF-001</t>
-        </is>
-      </c>
-      <c r="E4" s="84" t="inlineStr">
-        <is>
-          <t>TC-01</t>
-        </is>
-      </c>
-      <c r="F4" s="83" t="inlineStr">
+      <c r="D4" s="79" t="inlineStr">
+        <is>
+          <t>CRF-003</t>
+        </is>
+      </c>
+      <c r="E4" s="78" t="inlineStr">
+        <is>
+          <t>TC-03</t>
+        </is>
+      </c>
+      <c r="F4" s="78" t="inlineStr">
         <is>
           <t>26/02/2026</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="83" t="inlineStr">
-        <is>
-          <t>Modify Location Details Before Submission</t>
-        </is>
-      </c>
-      <c r="C5" s="83" t="inlineStr">
+      <c r="A5" s="78" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="B5" s="79" t="inlineStr">
+        <is>
+          <t>Validate Mobile Number length constraint (9 digits)</t>
+        </is>
+      </c>
+      <c r="C5" s="78" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D5" s="84" t="inlineStr">
-        <is>
-          <t>CRF-002</t>
-        </is>
-      </c>
-      <c r="E5" s="84" t="inlineStr">
-        <is>
-          <t>TC-02</t>
-        </is>
-      </c>
-      <c r="F5" s="83" t="inlineStr">
+      <c r="D5" s="79" t="inlineStr">
+        <is>
+          <t>CRF-004</t>
+        </is>
+      </c>
+      <c r="E5" s="78" t="inlineStr">
+        <is>
+          <t>TC-04</t>
+        </is>
+      </c>
+      <c r="F5" s="78" t="inlineStr">
         <is>
           <t>26/02/2026</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="83" t="inlineStr">
-        <is>
-          <t>Prevent progression with Empty required fields (Step 1)</t>
-        </is>
-      </c>
-      <c r="C6" s="83" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D6" s="84" t="inlineStr">
-        <is>
-          <t>CRF-003</t>
-        </is>
-      </c>
-      <c r="E6" s="84" t="inlineStr">
-        <is>
-          <t>TC-03</t>
-        </is>
-      </c>
-      <c r="F6" s="83" t="inlineStr">
+      <c r="A6" s="78" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="B6" s="79" t="inlineStr">
+        <is>
+          <t>Validate Email Format formatting (missing `@`)</t>
+        </is>
+      </c>
+      <c r="C6" s="78" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D6" s="79" t="inlineStr">
+        <is>
+          <t>CRF-005</t>
+        </is>
+      </c>
+      <c r="E6" s="78" t="inlineStr">
+        <is>
+          <t>TC-05</t>
+        </is>
+      </c>
+      <c r="F6" s="78" t="inlineStr">
         <is>
           <t>26/02/2026</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="83" t="inlineStr">
-        <is>
-          <t>Validate Mobile Number length constraint (9 digits)</t>
-        </is>
-      </c>
-      <c r="C7" s="83" t="inlineStr">
+      <c r="A7" s="78" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="B7" s="79" t="inlineStr">
+        <is>
+          <t>Prevent submission with Empty required fields (Step 2)</t>
+        </is>
+      </c>
+      <c r="C7" s="78" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D7" s="84" t="inlineStr">
-        <is>
-          <t>CRF-004</t>
-        </is>
-      </c>
-      <c r="E7" s="84" t="inlineStr">
-        <is>
-          <t>TC-04</t>
-        </is>
-      </c>
-      <c r="F7" s="83" t="inlineStr">
+      <c r="D7" s="79" t="inlineStr">
+        <is>
+          <t>CRF-006</t>
+        </is>
+      </c>
+      <c r="E7" s="78" t="inlineStr">
+        <is>
+          <t>TC-06</t>
+        </is>
+      </c>
+      <c r="F7" s="78" t="inlineStr">
         <is>
           <t>26/02/2026</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="83" t="inlineStr">
-        <is>
-          <t>Validate Email Format formatting (missing `@`)</t>
-        </is>
-      </c>
-      <c r="C8" s="83" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="D8" s="84" t="inlineStr">
-        <is>
-          <t>CRF-005</t>
-        </is>
-      </c>
-      <c r="E8" s="84" t="inlineStr">
-        <is>
-          <t>TC-05</t>
-        </is>
-      </c>
-      <c r="F8" s="83" t="inlineStr">
+      <c r="A8" s="78" t="inlineStr">
+        <is>
+          <t>7.0</t>
+        </is>
+      </c>
+      <c r="B8" s="79" t="inlineStr">
+        <is>
+          <t>Submit Current Date in "Date of Incident" field</t>
+        </is>
+      </c>
+      <c r="C8" s="78" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D8" s="79" t="inlineStr">
+        <is>
+          <t>CRF-007</t>
+        </is>
+      </c>
+      <c r="E8" s="78" t="inlineStr">
+        <is>
+          <t>TC-07</t>
+        </is>
+      </c>
+      <c r="F8" s="78" t="inlineStr">
         <is>
           <t>26/02/2026</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="83" t="inlineStr">
-        <is>
-          <t>Prevent submission with Empty required fields (Step 2)</t>
-        </is>
-      </c>
-      <c r="C9" s="83" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D9" s="84" t="inlineStr">
-        <is>
-          <t>CRF-006</t>
-        </is>
-      </c>
-      <c r="E9" s="84" t="inlineStr">
-        <is>
-          <t>TC-06</t>
-        </is>
-      </c>
-      <c r="F9" s="83" t="inlineStr">
+      <c r="A9" s="78" t="inlineStr">
+        <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="B9" s="79" t="inlineStr">
+        <is>
+          <t>Upload Unsupported File Type</t>
+        </is>
+      </c>
+      <c r="C9" s="78" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D9" s="79" t="inlineStr">
+        <is>
+          <t>CRF-008</t>
+        </is>
+      </c>
+      <c r="E9" s="78" t="inlineStr">
+        <is>
+          <t>TC-08</t>
+        </is>
+      </c>
+      <c r="F9" s="78" t="inlineStr">
         <is>
           <t>26/02/2026</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="83" t="inlineStr">
-        <is>
-          <t>Submit Current Date in "Date of Incident" field</t>
-        </is>
-      </c>
-      <c r="C10" s="83" t="inlineStr">
+      <c r="A10" s="78" t="inlineStr">
+        <is>
+          <t>9.0</t>
+        </is>
+      </c>
+      <c r="B10" s="79" t="inlineStr">
+        <is>
+          <t>Test phone number length exceeding 9 digits (Boundary)</t>
+        </is>
+      </c>
+      <c r="C10" s="78" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D10" s="84" t="inlineStr">
-        <is>
-          <t>CRF-007</t>
-        </is>
-      </c>
-      <c r="E10" s="84" t="inlineStr">
-        <is>
-          <t>TC-07</t>
-        </is>
-      </c>
-      <c r="F10" s="83" t="inlineStr">
+      <c r="D10" s="79" t="inlineStr">
+        <is>
+          <t>CRF-009</t>
+        </is>
+      </c>
+      <c r="E10" s="78" t="inlineStr">
+        <is>
+          <t>TC-09</t>
+        </is>
+      </c>
+      <c r="F10" s="78" t="inlineStr">
         <is>
           <t>26/02/2026</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="83" t="inlineStr">
-        <is>
-          <t>Upload Unsupported File Type</t>
-        </is>
-      </c>
-      <c r="C11" s="83" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D11" s="84" t="inlineStr">
-        <is>
-          <t>CRF-008</t>
-        </is>
-      </c>
-      <c r="E11" s="84" t="inlineStr">
-        <is>
-          <t>TC-08</t>
-        </is>
-      </c>
-      <c r="F11" s="83" t="inlineStr">
+      <c r="A11" s="78" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="B11" s="79" t="inlineStr">
+        <is>
+          <t>Test extremely long input for Name/Surname (Boundary)</t>
+        </is>
+      </c>
+      <c r="C11" s="78" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="D11" s="79" t="inlineStr">
+        <is>
+          <t>CRF-010</t>
+        </is>
+      </c>
+      <c r="E11" s="78" t="inlineStr">
+        <is>
+          <t>TC-10</t>
+        </is>
+      </c>
+      <c r="F11" s="78" t="inlineStr">
         <is>
           <t>26/02/2026</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="83" t="inlineStr">
-        <is>
-          <t>Test phone number length exceeding 9 digits (Boundary)</t>
-        </is>
-      </c>
-      <c r="C12" s="83" t="inlineStr">
+      <c r="A12" s="78" t="inlineStr">
+        <is>
+          <t>11.0</t>
+        </is>
+      </c>
+      <c r="B12" s="79" t="inlineStr">
+        <is>
+          <t>Automated Catch of "Future Date" Rejection on Current Date</t>
+        </is>
+      </c>
+      <c r="C12" s="78" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D12" s="84" t="inlineStr">
-        <is>
-          <t>CRF-009</t>
-        </is>
-      </c>
-      <c r="E12" s="84" t="inlineStr">
-        <is>
-          <t>TC-09</t>
-        </is>
-      </c>
-      <c r="F12" s="83" t="inlineStr">
-        <is>
-          <t>26/02/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="83" t="inlineStr">
-        <is>
-          <t>Test extremely long input for Name/Surname (Boundary)</t>
-        </is>
-      </c>
-      <c r="C13" s="83" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-      <c r="D13" s="84" t="inlineStr">
-        <is>
-          <t>CRF-010</t>
-        </is>
-      </c>
-      <c r="E13" s="84" t="inlineStr">
-        <is>
-          <t>TC-10</t>
-        </is>
-      </c>
-      <c r="F13" s="83" t="inlineStr">
-        <is>
-          <t>26/02/2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="83" t="inlineStr">
-        <is>
-          <t>Automated Catch of "Future Date" Rejection on Current Date</t>
-        </is>
-      </c>
-      <c r="C14" s="83" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D14" s="84" t="inlineStr">
+      <c r="D12" s="79" t="inlineStr">
         <is>
           <t>CRF-011</t>
         </is>
       </c>
-      <c r="E14" s="84" t="inlineStr">
+      <c r="E12" s="78" t="inlineStr">
         <is>
           <t>TC-11</t>
         </is>
       </c>
-      <c r="F14" s="83" t="inlineStr">
+      <c r="F12" s="78" t="inlineStr">
         <is>
           <t>26/02/2026</t>
         </is>
@@ -1314,13 +1309,58 @@
     <mergeCell ref="G7:J7"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="F10:F24" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
+    <dataValidation sqref="F10:F15" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
       <formula1>"Pass,Fail,Blocked,Not Executed,In progress,Retest,Deferred"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1" gridLines="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
+  <pageSetup orientation="landscape" fitToHeight="0" pageOrder="overThenDown" cellComments="atEnd"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="37.88" customWidth="1" style="77" min="1" max="1"/>
+    <col width="38.25" customWidth="1" style="77" min="2" max="2"/>
+    <col width="37.88" customWidth="1" style="77" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Automation Framework &amp; Tools Used</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Automation Architecture</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="78" t="inlineStr">
+        <is>
+          <t>Playwright (TypeScript/Node.js). Faster, reliable, auto-waits, native cross-browser.</t>
+        </is>
+      </c>
+      <c r="B2" s="78" t="inlineStr">
+        <is>
+          <t>tests/, pages/, data/ separated structure following POM.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>